<commit_message>
Add D14 to the workbook Decision Log
Mirrors the repository-visibility decision into the PRD workbook and
refreshes the Progress Log. Completes the workbook update deferred in
77f8cd1, which was blocked by an Excel file lock.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Raymund_Portfolio_PRD_Progress_Tracker.xlsx
+++ b/Raymund_Portfolio_PRD_Progress_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://gdslink-my.sharepoint.com/personal/raymund_bermudes_gdslinkasia_com/Documents/Documents/Rr/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="36" documentId="11_3FA3112190F2E404F161B51768A2211586063D4F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{42782C79-B455-4D65-B076-A4E8E069D3AF}"/>
+  <xr:revisionPtr revIDLastSave="49" documentId="11_3FA3112190F2E404F161B51768A2211586063D4F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CB9B05CB-FA39-42E7-B12B-FECF8C0F6298}"/>
   <bookViews>
     <workbookView xWindow="2304" yWindow="2304" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1452" uniqueCount="976">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1460" uniqueCount="984">
   <si>
     <t>Portfolio Project PRD &amp; Progress Tracker</t>
   </si>
@@ -2956,16 +2956,40 @@
     <t>Environment gate + D1-D13 approval + blockers cleared</t>
   </si>
   <si>
-    <t>Gate now PASSES: Node v24.19.0, npm 11.17.0, npm ping PONG, git 2.35.1, no proxy or TLS interception. All D1-D13 settled (11 as recommended; D9 and D13 amended). Stray home-level .git confirmed gone; git init -b main run inside the project folder with .gitignore written before any commit - git status shows 5 files, none from the user profile. No commit made yet.</t>
-  </si>
-  <si>
-    <t>B1 and B2 CLOSED. Two new open items: B5 - the project sits in a syncing corporate OneDrive folder, so node_modules will cause sync thrash and EPERM/EBUSY install failures once npm install runs; recommend relocating outside OneDrive before CHUNK 01. B6 - git user.email is the work address raymund.bermudes@gdslinkasia.com, which would be permanent and public in the commit history of a personal portfolio; set a repo-local identity before the first commit.</t>
-  </si>
-  <si>
-    <t>Owner decides B5 (project location) and B6 (commit identity), then CHUNK 01. CHUNK 00 needs neither and is the critical path.</t>
-  </si>
-  <si>
     <t>Ready to start</t>
+  </si>
+  <si>
+    <t>Raymund Ryan Bermudes</t>
+  </si>
+  <si>
+    <t>D14</t>
+  </si>
+  <si>
+    <t>GitHub repository visibility</t>
+  </si>
+  <si>
+    <t>Public repo; public with planning docs excluded; public with docs sanitised; private repo</t>
+  </si>
+  <si>
+    <t>PRIVATE repository</t>
+  </si>
+  <si>
+    <t>Not anticipated in the discovery report - raised when the first commit was prepared. A scan of the four planning documents found CTBC, CASECenter and SBC named throughout (CLAUDE.md, HANDOFF.md, PHASE-1-DISCOVERY.md and this workbook), and PHASE-1-DISCOVERY.md states that the SBC engagement involved security remediation - the exact association D5 places at Abstracted tier. A public repository would publish what D5 forbids, and git history is permanent: deleting files later does not remove them from history, existing clones or cached views. Vercel deploys from a private repo on the Hobby plan with no change to the site.</t>
+  </si>
+  <si>
+    <t>CRITICAL and IRREVERSIBLE if wrong. Never make this repo public without first rewriting history. Repo privacy does NOT relax D5 for the published site, and Vercel preview deployments remain publicly addressable - confirm preview protection at CHUNK 01.</t>
+  </si>
+  <si>
+    <t>DECIDED by owner 2026-09-22 - Private</t>
+  </si>
+  <si>
+    <t>Gate now PASSES: Node v24.19.0, npm 11.17.0, npm ping PONG, git 2.35.1, no proxy or TLS interception. All D1-D13 settled (11 as recommended; D9 and D13 amended), plus new D14. Stray home-level .git confirmed gone; git init -b main run inside the project folder; .gitignore written before any commit; repo-local user.email set to the GitHub noreply address with global config untouched. Commits ad51196 (planning artefacts) and 77f8cd1 (D14 + blockers closed).</t>
+  </si>
+  <si>
+    <t>B1, B2, B5 and B6 all CLOSED. New decision D14 raised and settled: a pre-commit scan found client names throughout the planning docs, so the GitHub repository must be PRIVATE. Remaining OneDrive mitigation: exclude node_modules from sync once CHUNK 01 creates it, and suspect OneDrive first if npm install fails with EPERM or EBUSY.</t>
+  </si>
+  <si>
+    <t>Owner creates an empty PRIVATE GitHub repo and a Vercel account; then CHUNK 01. CHUNK 00 needs neither and remains the critical path.</t>
   </si>
 </sst>
 </file>
@@ -3084,7 +3108,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -3114,6 +3138,7 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3448,7 +3473,7 @@
         <v>3</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>4</v>
+        <v>973</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
@@ -4000,19 +4025,19 @@
         <v>971</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>972</v>
+        <v>981</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>970</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>973</v>
+        <v>982</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>974</v>
+        <v>983</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>975</v>
+        <v>972</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
@@ -4063,7 +4088,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -4438,6 +4463,32 @@
       </c>
       <c r="H14" s="4" t="s">
         <v>966</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A15" s="11" t="s">
+        <v>555</v>
+      </c>
+      <c r="B15" t="s">
+        <v>974</v>
+      </c>
+      <c r="C15" t="s">
+        <v>975</v>
+      </c>
+      <c r="D15" t="s">
+        <v>976</v>
+      </c>
+      <c r="E15" t="s">
+        <v>977</v>
+      </c>
+      <c r="F15" t="s">
+        <v>978</v>
+      </c>
+      <c r="G15" t="s">
+        <v>979</v>
+      </c>
+      <c r="H15" t="s">
+        <v>980</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Record CHUNK 01 progress and add dev-server launch config
- HANDOFF.md: CHUNK 01 scope, what was verified, what remains before it can
  be marked Complete; Astro 7.3.3 and its >=22.12.0 Node floor recorded as
  verified facts rather than assumptions
- Workbook Progress Log: CHUNK 01 In Progress
- .claude/launch.json: dev server entry, invoking Astro through node directly
  because npm is not on PATH in the tooling environment

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Raymund_Portfolio_PRD_Progress_Tracker.xlsx
+++ b/Raymund_Portfolio_PRD_Progress_Tracker.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://gdslink-my.sharepoint.com/personal/raymund_bermudes_gdslinkasia_com/Documents/Documents/Rr/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RaymundBermudes\OneDrive - GDS Link, LLC\Documents\Rr\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="49" documentId="11_3FA3112190F2E404F161B51768A2211586063D4F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CB9B05CB-FA39-42E7-B12B-FECF8C0F6298}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD11F8FE-0DB8-4702-B965-22DAC0583F0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2304" yWindow="2304" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1460" uniqueCount="984">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1460" uniqueCount="983">
   <si>
     <t>Portfolio Project PRD &amp; Progress Tracker</t>
   </si>
@@ -2950,15 +2950,6 @@
     <t>Not used - no engagement is published at Named tier</t>
   </si>
   <si>
-    <t>HANDOFF.md</t>
-  </si>
-  <si>
-    <t>Environment gate + D1-D13 approval + blockers cleared</t>
-  </si>
-  <si>
-    <t>Ready to start</t>
-  </si>
-  <si>
     <t>Raymund Ryan Bermudes</t>
   </si>
   <si>
@@ -2983,13 +2974,19 @@
     <t>DECIDED by owner 2026-09-22 - Private</t>
   </si>
   <si>
-    <t>Gate now PASSES: Node v24.19.0, npm 11.17.0, npm ping PONG, git 2.35.1, no proxy or TLS interception. All D1-D13 settled (11 as recommended; D9 and D13 amended), plus new D14. Stray home-level .git confirmed gone; git init -b main run inside the project folder; .gitignore written before any commit; repo-local user.email set to the GitHub noreply address with global config untouched. Commits ad51196 (planning artefacts) and 77f8cd1 (D14 + blockers closed).</t>
-  </si>
-  <si>
-    <t>B1, B2, B5 and B6 all CLOSED. New decision D14 raised and settled: a pre-commit scan found client names throughout the planning docs, so the GitHub repository must be PRIVATE. Remaining OneDrive mitigation: exclude node_modules from sync once CHUNK 01 creates it, and suspect OneDrive first if npm install fails with EPERM or EBUSY.</t>
-  </si>
-  <si>
-    <t>Owner creates an empty PRIVATE GitHub repo and a Vercel account; then CHUNK 01. CHUNK 00 needs neither and remains the critical path.</t>
+    <t>CHUNK 01 - project foundation + security headers</t>
+  </si>
+  <si>
+    <t>Environment gate PASSES (Node v24.19.0, npm 11.17.0, npm ping PONG). All D1-D14 settled. Repo re-rooted, .gitignore and commit identity set. CHUNK 01 scaffolded: Astro 7.3.3 static, TypeScript strict, @astrojs/check, engines node &gt;=22.12.0 (verified against the registry, not assumed). vercel.json carries CSP, HSTS, X-Content-Type-Options, Referrer-Policy, Permissions-Policy, X-Frame-Options, COOP, CORP and immutable caching for hashed assets. Astro build telemetry disabled. Placeholder home page with noindex. Tailwind, MDX and the real pages deliberately deferred to their own chunks.</t>
+  </si>
+  <si>
+    <t>Commits ad51196, 77f8cd1, ac73cdb, b1f806c</t>
+  </si>
+  <si>
+    <t>CHUNK 01 is NOT complete: the deploy is outstanding and needs a private GitHub repo URL from the owner. Security headers are therefore UNPROVEN - vercel.json has no effect on the dev server and must be verified against a live deployment. astro.config.mjs `site` is still commented out and CHUNK 15 cannot complete without it.</t>
+  </si>
+  <si>
+    <t>Owner supplies the private GitHub repo URL; push, import to Vercel (Hobby), set `site`, then verify headers against the deployment. CHUNK 02 (design system) and CHUNK 04 (content layer) are unblocked and can start in parallel. CHUNK 00 remains the critical path.</t>
   </si>
 </sst>
 </file>
@@ -3134,11 +3131,11 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3449,13 +3446,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
     </row>
     <row r="2" spans="1:5" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
@@ -3473,7 +3470,7 @@
         <v>3</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>973</v>
+        <v>970</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
@@ -4022,22 +4019,22 @@
         <v>96</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>971</v>
+        <v>978</v>
       </c>
       <c r="D5" s="2" t="s">
+        <v>979</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>980</v>
+      </c>
+      <c r="F5" s="2" t="s">
         <v>981</v>
       </c>
-      <c r="E5" s="2" t="s">
-        <v>970</v>
-      </c>
-      <c r="F5" s="2" t="s">
+      <c r="G5" s="2" t="s">
         <v>982</v>
       </c>
-      <c r="G5" s="2" t="s">
-        <v>983</v>
-      </c>
       <c r="H5" s="2" t="s">
-        <v>972</v>
+        <v>43</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
@@ -4466,29 +4463,29 @@
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A15" s="11" t="s">
+      <c r="A15" s="9" t="s">
         <v>555</v>
       </c>
       <c r="B15" t="s">
+        <v>971</v>
+      </c>
+      <c r="C15" t="s">
+        <v>972</v>
+      </c>
+      <c r="D15" t="s">
+        <v>973</v>
+      </c>
+      <c r="E15" t="s">
         <v>974</v>
       </c>
-      <c r="C15" t="s">
+      <c r="F15" t="s">
         <v>975</v>
       </c>
-      <c r="D15" t="s">
+      <c r="G15" t="s">
         <v>976</v>
       </c>
-      <c r="E15" t="s">
+      <c r="H15" t="s">
         <v>977</v>
-      </c>
-      <c r="F15" t="s">
-        <v>978</v>
-      </c>
-      <c r="G15" t="s">
-        <v>979</v>
-      </c>
-      <c r="H15" t="s">
-        <v>980</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Set canonical site URL; record live deployment and header verification
- astro.config.mjs: site set to the production origin. Canonical URLs, OG
  tags and the sitemap now have a real base; CHUNK 15 is unblocked.
- All nine security headers verified against a live HTTP response rather
  than against vercel.json. The dev server does not serve them, so
  localhost proves nothing.

Finding: Vercel preview and branch deployment URLs are public - both
returned HTTP 200 unauthenticated. Harmless while the site is a
placeholder, but from CHUNK 07 a draft case study on any branch would be
publicly readable before D5 clearance. Mitigation recorded: clearance is a
pre-commit gate, not a pre-merge one. Branch privacy is not a
confidentiality control.

Also noted: Vercel adds an Access-Control-Allow-Origin header we did not
set. Benign on a credential-free static site; flagged for CHUNK 16.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Raymund_Portfolio_PRD_Progress_Tracker.xlsx
+++ b/Raymund_Portfolio_PRD_Progress_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RaymundBermudes\OneDrive - GDS Link, LLC\Documents\Rr\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD11F8FE-0DB8-4702-B965-22DAC0583F0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1A649B4-0AE9-4B43-BDA5-79CDD1922589}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2304" yWindow="2304" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1460" uniqueCount="983">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1460" uniqueCount="984">
   <si>
     <t>Portfolio Project PRD &amp; Progress Tracker</t>
   </si>
@@ -2977,16 +2977,19 @@
     <t>CHUNK 01 - project foundation + security headers</t>
   </si>
   <si>
-    <t>Environment gate PASSES (Node v24.19.0, npm 11.17.0, npm ping PONG). All D1-D14 settled. Repo re-rooted, .gitignore and commit identity set. CHUNK 01 scaffolded: Astro 7.3.3 static, TypeScript strict, @astrojs/check, engines node &gt;=22.12.0 (verified against the registry, not assumed). vercel.json carries CSP, HSTS, X-Content-Type-Options, Referrer-Policy, Permissions-Policy, X-Frame-Options, COOP, CORP and immutable caching for hashed assets. Astro build telemetry disabled. Placeholder home page with noindex. Tailwind, MDX and the real pages deliberately deferred to their own chunks.</t>
-  </si>
-  <si>
-    <t>Commits ad51196, 77f8cd1, ac73cdb, b1f806c</t>
-  </si>
-  <si>
-    <t>CHUNK 01 is NOT complete: the deploy is outstanding and needs a private GitHub repo URL from the owner. Security headers are therefore UNPROVEN - vercel.json has no effect on the dev server and must be verified against a live deployment. astro.config.mjs `site` is still commented out and CHUNK 15 cannot complete without it.</t>
-  </si>
-  <si>
-    <t>Owner supplies the private GitHub repo URL; push, import to Vercel (Hobby), set `site`, then verify headers against the deployment. CHUNK 02 (design system) and CHUNK 04 (content layer) are unblocked and can start in parallel. CHUNK 00 remains the critical path.</t>
+    <t>CHUNK 01 built and DEPLOYED. Astro 7.3.3 static, TypeScript strict, engines node &gt;=22.12.0 (verified against the registry). Live at https://raymundbermudes.vercel.app on the Hobby plan from the private repo rrcreations69/ClaudePortfolio, deployed by the personal account. All NINE security headers verified against a real HTTP response from the live deployment, not against vercel.json: CSP, HSTS, X-Content-Type-Options, Referrer-Policy, Permissions-Policy, X-Frame-Options, COOP, CORP, X-DNS-Prefetch-Control. Output is zero JavaScript, 2,387 bytes. Astro build telemetry disabled. site set in astro.config.mjs.</t>
+  </si>
+  <si>
+    <t>https://raymundbermudes.vercel.app</t>
+  </si>
+  <si>
+    <t>FINDING: Vercel preview/branch deployment URLs are PUBLIC - both alternate URLs returned HTTP 200 unauthenticated. Harmless now (placeholder content) but a confidentiality risk from CHUNK 07: a draft case study pushed to any branch is publicly readable before D5 clearance. MITIGATION (plan-independent): make confidentiality clearance a PRE-COMMIT gate, never rely on branch privacy. Also noted: Vercel adds Access-Control-Allow-Origin: * which we did not set - benign on a credential-free static site, flagged for CHUNK 16 review.</t>
+  </si>
+  <si>
+    <t>Push the `site` config commit and confirm the redeploy, then CHUNK 01 is Complete. CHUNK 02 (design system) and CHUNK 04 (content layer) are unblocked. CHUNK 00 remains the critical path.</t>
+  </si>
+  <si>
+    <t>Review</t>
   </si>
 </sst>
 </file>
@@ -4034,7 +4037,7 @@
         <v>982</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>43</v>
+        <v>983</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Tracker: D31-D33, CG-02 and CG-12 closed
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Raymund_Portfolio_PRD_Progress_Tracker.xlsx
+++ b/Raymund_Portfolio_PRD_Progress_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://gdslink-my.sharepoint.com/personal/raymund_bermudes_gdslinkasia_com/Documents/Documents/Rr/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="444" documentId="13_ncr:1_{E42DE829-FADD-499D-AC40-0688BE14A681}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5609FDCD-889A-4FCF-B514-CAECBA49139A}"/>
+  <xr:revisionPtr revIDLastSave="479" documentId="13_ncr:1_{E42DE829-FADD-499D-AC40-0688BE14A681}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BC2CE1DC-2AE1-4B04-8F07-DFB7DE1AF9E2}"/>
   <bookViews>
     <workbookView xWindow="2304" yWindow="2304" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1783" uniqueCount="1224">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1812" uniqueCount="1249">
   <si>
     <t>Portfolio Project PRD &amp; Progress Tracker</t>
   </si>
@@ -3238,9 +3238,6 @@
     <t>Case study 2 - CASECenter policy system delivery (current Solutions Analyst role). DECIDED 2026-09-23. NOTE: this row previously read "SBC security work", which was mis-scoped - SBC is a third mobile maintenance engagement (older app, Java), not separate security work.</t>
   </si>
   <si>
-    <t>Open - BLOCKING. Engagement chosen (CASECenter). Skeleton drafted in notes/case-study-2-DRAFT.md; all ten sections still need Raymund's account.</t>
-  </si>
-  <si>
     <t>Drafted case study skeletons for BOTH case studies into notes/, against the ten Sheet 06 sections. Every drafted line traces to a quoted statement; everything else marked [CONTENT REQUIRED]. Method: draft-and-correct rather than open questioning. Case study 1 (VAPT, abstracted tier): decisions 1 and 2 answered - the remediation was TRIAGE, not a blanket no-upgrade constraint. Raymund upgraded the libraries that could move without breaking the base code and closed the rest in the application's own code. That is a judgement story rather than a constraint story, and materially stronger. His earlier "cannot update any library" was shorthand, not a contradiction; the case study must use the accurate version. Case study 2 (CASECenter, sectoral tier): engagement chosen; closes the gap between the new positioning (D15, Enterprise Systems Developer) and the evidence, which was otherwise all Android.</t>
   </si>
   <si>
@@ -3664,9 +3661,6 @@
     <t>CLOSED 2026-09-24 - NO screenshots are cleared and NONE are used anywhere on the site. The default assumption (none) stands as the permanent answer.</t>
   </si>
   <si>
-    <t>Partially closed 2026-09-24 - case study 1 needed NO architecture figure: its story is dependency judgement, not topology, and a diagram would have added identifying detail for no benefit. Re-open for case study 2 if the policy system needs one.</t>
-  </si>
-  <si>
     <t>CLOSED 2026-09-22 (D9) - the site stays on *.vercel.app permanently. No custom domain. This row was stale.</t>
   </si>
   <si>
@@ -3710,6 +3704,87 @@
   </si>
   <si>
     <t>Open - ADDED 2026-09-24. This gap was being rendered on /about as a visible [CONTENT REQUIRED] but was never tracked on this sheet. Nobody but the owner can write it; a generated version reads exactly like one.</t>
+  </si>
+  <si>
+    <t>D31</t>
+  </si>
+  <si>
+    <t>Case study 2 publishes at abstracted, NOT the sectoral the skeleton proposed</t>
+  </si>
+  <si>
+    <t>(a) sectoral - sector, scale and geography, no name; (b) abstracted - class of problem only</t>
+  </si>
+  <si>
+    <t>(b) abstracted</t>
+  </si>
+  <si>
+    <t>GDS Link Asia serves a small, named set of credit-decisioning clients. At sectoral, "a Taiwanese bank" or "a Philippine commercial bank" is shortlistable in one guess - and a tier that only FEELS protective is worse than one that is, because it licenses more detail on a false assumption. abstracted costs nothing here: the story is requirements, policy logic, UAT and sign-off, none of which need the client identity. CASECenter and GDS Link Asia stay nameable per D18 - the tier governs the CLIENT, not the tool.</t>
+  </si>
+  <si>
+    <t>Medium. Overrides the skeleton default in notes/case-study-2-DRAFT.md.</t>
+  </si>
+  <si>
+    <t>DECIDED by owner 2026-09-24</t>
+  </si>
+  <si>
+    <t>D32</t>
+  </si>
+  <si>
+    <t>Case study 2 ships as a SHORT ENTRY, not a full ten-section case study</t>
+  </si>
+  <si>
+    <t>(a) Full nine-question interview; (b) short entry, five questions; (c) ship with one case study only</t>
+  </si>
+  <si>
+    <t>(b) Short entry</t>
+  </si>
+  <si>
+    <t>Owner pushed back on depth: "WHY DO WE GO DEEP ON MY THINGS I DID IN MY WORK? I JUST NEED A SHOWCASE OF MY CV". The trade-off was stated once and accepted: the CV-showcase job is ALREADY done by /about, the home page and the PDF, so the Work section is the only part not already in the CV - which is why depth lives there. A short entry closes the Android-only evidence gap at a fraction of the effort.</t>
+  </si>
+  <si>
+    <t>Medium. Schema forcing functions still apply and were NOT skipped - clientDescriptor, problem, myRole and outcome are all .min(1). What was dropped is the ten-section Sheet 06 body: four short sections instead of ten. Cost: no Lessons section, because that question was not asked in the short scope and nothing was available to source it from.</t>
+  </si>
+  <si>
+    <t>D33</t>
+  </si>
+  <si>
+    <t>The stages field is rendered, via a new StageCoverage component</t>
+  </si>
+  <si>
+    <t>(a) Leave stages unrendered; (b) render it; (c) delete it from the schema</t>
+  </si>
+  <si>
+    <t>(b) Render it</t>
+  </si>
+  <si>
+    <t>stages had been in the schema since CHUNK 04 and rendered NOWHERE, and the schema comment wrongly claimed it "drives the Delivery Thread rail" - the rail is built from rendered headings. So "covered seven of seven stages" was a claim stored in a file nobody reads, and the central argument for having a Delivery Thread at all was invisible to a recruiter. UNCOVERED stages stay visible deliberately: case study 1 renders 4 of 7 with three hollow rings, and that honesty is what makes the 7 of 7 beside it worth believing.</t>
+  </si>
+  <si>
+    <t>Medium. New no-JS component in the case study header. Coverage conveyed THREE ways - marker shape, token colour, and visually-hidden covered/not-covered text - never by colour alone. No opacity is used to dim: opacity has broken AAA twice on this site and axe cannot detect it. Measured: light 7.77/18.47/8.13, dark 8.07/17.51, all AAA; no overflow at 320px.</t>
+  </si>
+  <si>
+    <t>DECIDED by Claude 2026-09-24, reported to owner and approved</t>
+  </si>
+  <si>
+    <t>CLOSED 2026-09-24 - published as src/content/work/delivering-from-an-unfinished-requirements-document.mdx at abstracted tier (D31), short-entry scope (D32). Sourced entirely from five owner answers plus one follow-up. CONFIDENTIALITY: his first answer named the business function, which is the SAME one deliberately removed from case study 1 - the two are two halves of one system (Android field capture syncing to the CASECenter side). Publishing it here would have handed back what case study 1 withheld: neither page leaks alone, both leak together. He chose generic. Audited on built HTML - zero occurrences.</t>
+  </si>
+  <si>
+    <t>CLOSED 2026-09-24 - NEITHER case study needed an architecture figure. Case study 1 is dependency judgement, not topology; case study 2 is delivery process. In both, a diagram would have added identifying detail for no engineering benefit. ArchitectureFigure remains available if a future entry needs one.</t>
+  </si>
+  <si>
+    <t>CHUNK 07 - case study 2 published, and stages made visible</t>
+  </si>
+  <si>
+    <t>Second Work entry live: "Push back before you build: delivering from an unfinished requirements document", 2024-2025, abstracted tier, SEVEN of seven delivery stages. It is the current role and it covers requirements and UAT, neither of which case study 1 touches - closing the gap where the positioning claimed enterprise systems delivery while every published piece of evidence was Android from the PREVIOUS role. Separately, the stages field was found to render nowhere despite being in the schema since CHUNK 04; new StageCoverage component now renders it (D33).</t>
+  </si>
+  <si>
+    <t>npm run verify exit 0, 22/22 guards, astro check 0/0/1, 8 pages. /work lists both entries. Case study pages render "4 of 7" and "7 of 7". Contrast measured in-browser: light 7.77/18.47/8.13, dark 8.07/17.51 - all AAA, computed opacity 1 throughout. No horizontal overflow at 320px.</t>
+  </si>
+  <si>
+    <t>CONFIDENTIALITY CATCH: the owner's first answer named the business function, the same one deliberately stripped from case study 1 on his own instruction. The two entries are two halves of one system, so publishing it would have re-identified what case study 1 withheld - a mosaic disclosure that neither page commits alone. Flagged, he chose generic, audited clean on built HTML. SOURCING: UAT and client sign-off were withheld from the first draft because he had said only "testing" and "went live"; he then confirmed DEV -&gt; UAT -&gt; Prod with sign-off, so both are now claimed. No Lessons section - not asked in the short scope, so nothing to source it from. No number anywhere.</t>
+  </si>
+  <si>
+    <t>Only TWO content items remain: the About story (CG-15) and the CV PDF file (CG-04). Then push, verify CHUNKS 14-16 against production, delete /styleguide, re-run Sheet 13 recruiter test.</t>
   </si>
 </sst>
 </file>
@@ -4330,10 +4405,10 @@
         <v>497</v>
       </c>
       <c r="D2" s="2" t="s">
+        <v>1096</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>1097</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>1098</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
@@ -4347,10 +4422,10 @@
         <v>500</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>1097</v>
+        <v>1096</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>1099</v>
+        <v>1098</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
@@ -4364,10 +4439,10 @@
         <v>503</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>1097</v>
+        <v>1096</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>1100</v>
+        <v>1099</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
@@ -4381,10 +4456,10 @@
         <v>505</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>1097</v>
+        <v>1096</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>1101</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
@@ -4398,10 +4473,10 @@
         <v>507</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>1097</v>
+        <v>1096</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>1102</v>
+        <v>1101</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
@@ -4415,10 +4490,10 @@
         <v>509</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>1097</v>
+        <v>1096</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>1103</v>
+        <v>1102</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="273.60000000000002" x14ac:dyDescent="0.3">
@@ -4432,10 +4507,10 @@
         <v>512</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>1097</v>
+        <v>1096</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>1104</v>
+        <v>1103</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="345.6" x14ac:dyDescent="0.3">
@@ -4449,10 +4524,10 @@
         <v>514</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>1097</v>
+        <v>1096</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>1105</v>
+        <v>1104</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="216" x14ac:dyDescent="0.3">
@@ -4466,10 +4541,10 @@
         <v>516</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>1097</v>
+        <v>1096</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>1143</v>
+        <v>1142</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="345.6" x14ac:dyDescent="0.3">
@@ -4483,10 +4558,10 @@
         <v>518</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>1097</v>
+        <v>1096</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>1139</v>
+        <v>1138</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="115.2" x14ac:dyDescent="0.3">
@@ -4500,10 +4575,10 @@
         <v>520</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>1097</v>
+        <v>1096</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>1138</v>
+        <v>1137</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="158.4" x14ac:dyDescent="0.3">
@@ -4517,10 +4592,10 @@
         <v>522</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>1097</v>
+        <v>1096</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="360" x14ac:dyDescent="0.3">
@@ -4534,10 +4609,10 @@
         <v>524</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>1097</v>
+        <v>1096</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>1136</v>
+        <v>1135</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="230.4" x14ac:dyDescent="0.3">
@@ -4551,10 +4626,10 @@
         <v>526</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>1097</v>
+        <v>1096</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>1135</v>
+        <v>1134</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="244.8" x14ac:dyDescent="0.3">
@@ -4568,10 +4643,10 @@
         <v>528</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>1097</v>
+        <v>1096</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>1134</v>
+        <v>1133</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="316.8" x14ac:dyDescent="0.3">
@@ -4585,10 +4660,10 @@
         <v>530</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>1097</v>
+        <v>1096</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>1133</v>
+        <v>1132</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="216" x14ac:dyDescent="0.3">
@@ -4602,10 +4677,10 @@
         <v>532</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>1097</v>
+        <v>1096</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>1142</v>
+        <v>1141</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="230.4" x14ac:dyDescent="0.3">
@@ -4619,10 +4694,10 @@
         <v>535</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>1097</v>
+        <v>1096</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="244.8" x14ac:dyDescent="0.3">
@@ -4636,10 +4711,10 @@
         <v>537</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>1097</v>
+        <v>1096</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>1140</v>
+        <v>1139</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
@@ -4653,10 +4728,10 @@
         <v>540</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>1124</v>
+        <v>1123</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>1144</v>
+        <v>1143</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="158.4" x14ac:dyDescent="0.3">
@@ -4670,10 +4745,10 @@
         <v>542</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>1124</v>
+        <v>1123</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>1145</v>
+        <v>1144</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
@@ -4687,10 +4762,10 @@
         <v>544</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>1124</v>
+        <v>1123</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>1146</v>
+        <v>1145</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="115.2" x14ac:dyDescent="0.3">
@@ -4704,10 +4779,10 @@
         <v>546</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>1122</v>
+        <v>1121</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>1147</v>
+        <v>1146</v>
       </c>
     </row>
   </sheetData>
@@ -4717,7 +4792,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:H24"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -4980,10 +5055,10 @@
         <v>997</v>
       </c>
       <c r="F10" s="11" t="s">
+        <v>1070</v>
+      </c>
+      <c r="G10" s="11" t="s">
         <v>1071</v>
-      </c>
-      <c r="G10" s="11" t="s">
-        <v>1072</v>
       </c>
       <c r="H10" s="11" t="s">
         <v>34</v>
@@ -5000,16 +5075,16 @@
         <v>1059</v>
       </c>
       <c r="D11" s="11" t="s">
+        <v>1066</v>
+      </c>
+      <c r="E11" s="11" t="s">
         <v>1067</v>
       </c>
-      <c r="E11" s="11" t="s">
+      <c r="F11" s="11" t="s">
         <v>1068</v>
       </c>
-      <c r="F11" s="11" t="s">
+      <c r="G11" s="11" t="s">
         <v>1069</v>
-      </c>
-      <c r="G11" s="11" t="s">
-        <v>1070</v>
       </c>
       <c r="H11" s="11" t="s">
         <v>42</v>
@@ -5017,103 +5092,103 @@
     </row>
     <row r="12" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A12" s="10" t="s">
-        <v>1075</v>
+        <v>1074</v>
       </c>
       <c r="B12" s="11" t="s">
         <v>94</v>
       </c>
       <c r="C12" s="11" t="s">
+        <v>1075</v>
+      </c>
+      <c r="D12" s="11" t="s">
         <v>1076</v>
       </c>
-      <c r="D12" s="11" t="s">
+      <c r="E12" s="11" t="s">
         <v>1077</v>
       </c>
-      <c r="E12" s="11" t="s">
+      <c r="F12" s="11" t="s">
         <v>1078</v>
       </c>
-      <c r="F12" s="11" t="s">
+      <c r="G12" s="11" t="s">
         <v>1079</v>
       </c>
-      <c r="G12" s="11" t="s">
-        <v>1080</v>
-      </c>
       <c r="H12" s="11" t="s">
-        <v>1074</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A13" s="10" t="s">
-        <v>1075</v>
+        <v>1074</v>
       </c>
       <c r="B13" s="11" t="s">
         <v>94</v>
       </c>
       <c r="C13" s="11" t="s">
+        <v>1081</v>
+      </c>
+      <c r="D13" s="11" t="s">
         <v>1082</v>
       </c>
-      <c r="D13" s="11" t="s">
+      <c r="E13" s="11" t="s">
         <v>1083</v>
       </c>
-      <c r="E13" s="11" t="s">
+      <c r="F13" s="11" t="s">
         <v>1084</v>
       </c>
-      <c r="F13" s="11" t="s">
+      <c r="G13" s="11" t="s">
         <v>1085</v>
       </c>
-      <c r="G13" s="11" t="s">
-        <v>1086</v>
-      </c>
       <c r="H13" s="11" t="s">
-        <v>1074</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A14" s="10" t="s">
-        <v>1075</v>
+        <v>1074</v>
       </c>
       <c r="B14" s="11" t="s">
         <v>94</v>
       </c>
       <c r="C14" s="11" t="s">
+        <v>1086</v>
+      </c>
+      <c r="D14" s="11" t="s">
         <v>1087</v>
       </c>
-      <c r="D14" s="11" t="s">
+      <c r="E14" s="11" t="s">
         <v>1088</v>
       </c>
-      <c r="E14" s="11" t="s">
+      <c r="F14" s="11" t="s">
         <v>1089</v>
       </c>
-      <c r="F14" s="11" t="s">
+      <c r="G14" s="11" t="s">
         <v>1090</v>
       </c>
-      <c r="G14" s="11" t="s">
-        <v>1091</v>
-      </c>
       <c r="H14" s="11" t="s">
-        <v>1074</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A15" s="10" t="s">
-        <v>1075</v>
+        <v>1074</v>
       </c>
       <c r="B15" s="11" t="s">
         <v>141</v>
       </c>
       <c r="C15" s="11" t="s">
+        <v>1091</v>
+      </c>
+      <c r="D15" s="11" t="s">
         <v>1092</v>
       </c>
-      <c r="D15" s="11" t="s">
+      <c r="E15" s="11" t="s">
         <v>1093</v>
       </c>
-      <c r="E15" s="11" t="s">
+      <c r="F15" s="11" t="s">
         <v>1094</v>
       </c>
-      <c r="F15" s="11" t="s">
+      <c r="G15" s="11" t="s">
         <v>1095</v>
-      </c>
-      <c r="G15" s="11" t="s">
-        <v>1096</v>
       </c>
       <c r="H15" s="11" t="s">
         <v>34</v>
@@ -5121,25 +5196,25 @@
     </row>
     <row r="16" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A16" s="10" t="s">
-        <v>1075</v>
+        <v>1074</v>
       </c>
       <c r="B16" s="11" t="s">
         <v>141</v>
       </c>
       <c r="C16" s="11" t="s">
+        <v>1105</v>
+      </c>
+      <c r="D16" s="11" t="s">
         <v>1106</v>
       </c>
-      <c r="D16" s="11" t="s">
+      <c r="E16" s="11" t="s">
         <v>1107</v>
       </c>
-      <c r="E16" s="11" t="s">
+      <c r="F16" s="11" t="s">
         <v>1108</v>
       </c>
-      <c r="F16" s="11" t="s">
+      <c r="G16" s="11" t="s">
         <v>1109</v>
-      </c>
-      <c r="G16" s="11" t="s">
-        <v>1110</v>
       </c>
       <c r="H16" s="11" t="s">
         <v>34</v>
@@ -5147,173 +5222,199 @@
     </row>
     <row r="17" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A17" s="10" t="s">
-        <v>1075</v>
+        <v>1074</v>
       </c>
       <c r="B17" s="11" t="s">
         <v>141</v>
       </c>
       <c r="C17" s="11" t="s">
+        <v>1110</v>
+      </c>
+      <c r="D17" s="11" t="s">
         <v>1111</v>
       </c>
-      <c r="D17" s="11" t="s">
+      <c r="E17" s="11" t="s">
         <v>1112</v>
       </c>
-      <c r="E17" s="11" t="s">
+      <c r="F17" s="11" t="s">
         <v>1113</v>
       </c>
-      <c r="F17" s="11" t="s">
+      <c r="G17" s="11" t="s">
         <v>1114</v>
       </c>
-      <c r="G17" s="11" t="s">
-        <v>1115</v>
-      </c>
       <c r="H17" s="11" t="s">
-        <v>1074</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A18" s="10" t="s">
-        <v>1075</v>
+        <v>1074</v>
       </c>
       <c r="B18" s="11" t="s">
         <v>141</v>
       </c>
       <c r="C18" s="11" t="s">
+        <v>1115</v>
+      </c>
+      <c r="D18" s="11" t="s">
         <v>1116</v>
       </c>
-      <c r="D18" s="11" t="s">
+      <c r="E18" s="11" t="s">
         <v>1117</v>
       </c>
-      <c r="E18" s="11" t="s">
+      <c r="F18" s="11" t="s">
         <v>1118</v>
       </c>
-      <c r="F18" s="11" t="s">
+      <c r="G18" s="11" t="s">
         <v>1119</v>
       </c>
-      <c r="G18" s="11" t="s">
-        <v>1120</v>
-      </c>
       <c r="H18" s="11" t="s">
-        <v>1074</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A19" s="10" t="s">
-        <v>1075</v>
+        <v>1074</v>
       </c>
       <c r="B19" s="11" t="s">
         <v>170</v>
       </c>
       <c r="C19" s="11" t="s">
+        <v>1147</v>
+      </c>
+      <c r="D19" s="11" t="s">
         <v>1148</v>
       </c>
-      <c r="D19" s="11" t="s">
+      <c r="E19" s="11" t="s">
         <v>1149</v>
       </c>
-      <c r="E19" s="11" t="s">
+      <c r="F19" s="11" t="s">
         <v>1150</v>
       </c>
-      <c r="F19" s="11" t="s">
+      <c r="G19" s="11" t="s">
         <v>1151</v>
       </c>
-      <c r="G19" s="11" t="s">
-        <v>1152</v>
-      </c>
       <c r="H19" s="11" t="s">
-        <v>1074</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A20" s="10" t="s">
-        <v>1075</v>
+        <v>1074</v>
       </c>
       <c r="B20" s="11" t="s">
         <v>39</v>
       </c>
       <c r="C20" s="11" t="s">
+        <v>1154</v>
+      </c>
+      <c r="D20" s="11" t="s">
         <v>1155</v>
       </c>
-      <c r="D20" s="11" t="s">
+      <c r="E20" s="11" t="s">
         <v>1156</v>
       </c>
-      <c r="E20" s="11" t="s">
+      <c r="F20" s="11" t="s">
         <v>1157</v>
       </c>
-      <c r="F20" s="11" t="s">
+      <c r="G20" s="11" t="s">
         <v>1158</v>
       </c>
-      <c r="G20" s="11" t="s">
-        <v>1159</v>
-      </c>
       <c r="H20" s="11" t="s">
-        <v>1074</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A21" s="10" t="s">
-        <v>1075</v>
+        <v>1074</v>
       </c>
       <c r="B21" s="11" t="s">
         <v>39</v>
       </c>
       <c r="C21" s="11" t="s">
+        <v>1213</v>
+      </c>
+      <c r="D21" s="11" t="s">
+        <v>1214</v>
+      </c>
+      <c r="E21" s="11" t="s">
         <v>1215</v>
       </c>
-      <c r="D21" s="11" t="s">
+      <c r="F21" s="11" t="s">
         <v>1216</v>
       </c>
-      <c r="E21" s="11" t="s">
+      <c r="G21" s="11" t="s">
         <v>1217</v>
-      </c>
-      <c r="F21" s="11" t="s">
-        <v>1218</v>
-      </c>
-      <c r="G21" s="11" t="s">
-        <v>1219</v>
       </c>
       <c r="H21" s="11" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A22" s="2"/>
-      <c r="B22" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="C22" s="2"/>
-      <c r="D22" s="2" t="s">
-        <v>569</v>
-      </c>
-      <c r="E22" s="2"/>
-      <c r="F22" s="2"/>
-      <c r="G22" s="2" t="s">
-        <v>570</v>
-      </c>
-      <c r="H22" s="2" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A22" s="10" t="s">
+        <v>1074</v>
+      </c>
+      <c r="B22" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="C22" s="11" t="s">
+        <v>1244</v>
+      </c>
+      <c r="D22" s="11" t="s">
+        <v>1245</v>
+      </c>
+      <c r="E22" s="11" t="s">
+        <v>1246</v>
+      </c>
+      <c r="F22" s="11" t="s">
+        <v>1247</v>
+      </c>
+      <c r="G22" s="11" t="s">
+        <v>1248</v>
+      </c>
+      <c r="H22" s="11" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A23" s="2"/>
       <c r="B23" s="2" t="s">
-        <v>170</v>
+        <v>141</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" s="2" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="E23" s="2"/>
       <c r="F23" s="2"/>
       <c r="G23" s="2" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
       <c r="H23" s="2" t="s">
         <v>48</v>
       </c>
     </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A24" s="2"/>
+      <c r="B24" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="C24" s="2"/>
+      <c r="D24" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="E24" s="2"/>
+      <c r="F24" s="2"/>
+      <c r="G24" s="2" t="s">
+        <v>572</v>
+      </c>
+      <c r="H24" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="H2:H23" xr:uid="{00000000-0002-0000-0A00-000000000000}">
+    <dataValidation type="list" allowBlank="1" sqref="H2:H24" xr:uid="{00000000-0002-0000-0A00-000000000000}">
       <formula1>"Not Started,In Progress,Blocked,Review,Complete,On Hold"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5323,7 +5424,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
-  <dimension ref="A1:H31"/>
+  <dimension ref="A1:H34"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -5965,25 +6066,25 @@
         <v>46289</v>
       </c>
       <c r="B25" t="s">
+        <v>1159</v>
+      </c>
+      <c r="C25" t="s">
         <v>1160</v>
       </c>
-      <c r="C25" t="s">
+      <c r="D25" t="s">
         <v>1161</v>
       </c>
-      <c r="D25" t="s">
+      <c r="E25" t="s">
         <v>1162</v>
       </c>
-      <c r="E25" t="s">
+      <c r="F25" t="s">
         <v>1163</v>
       </c>
-      <c r="F25" t="s">
+      <c r="G25" t="s">
         <v>1164</v>
       </c>
-      <c r="G25" t="s">
+      <c r="H25" t="s">
         <v>1165</v>
-      </c>
-      <c r="H25" t="s">
-        <v>1166</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.3">
@@ -5991,25 +6092,25 @@
         <v>46289</v>
       </c>
       <c r="B26" t="s">
+        <v>1166</v>
+      </c>
+      <c r="C26" t="s">
         <v>1167</v>
       </c>
-      <c r="C26" t="s">
+      <c r="D26" t="s">
         <v>1168</v>
       </c>
-      <c r="D26" t="s">
+      <c r="E26" t="s">
         <v>1169</v>
       </c>
-      <c r="E26" t="s">
+      <c r="F26" t="s">
         <v>1170</v>
       </c>
-      <c r="F26" t="s">
+      <c r="G26" t="s">
         <v>1171</v>
       </c>
-      <c r="G26" t="s">
+      <c r="H26" t="s">
         <v>1172</v>
-      </c>
-      <c r="H26" t="s">
-        <v>1173</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.3">
@@ -6017,25 +6118,25 @@
         <v>46289</v>
       </c>
       <c r="B27" t="s">
+        <v>1173</v>
+      </c>
+      <c r="C27" t="s">
         <v>1174</v>
       </c>
-      <c r="C27" t="s">
+      <c r="D27" t="s">
         <v>1175</v>
       </c>
-      <c r="D27" t="s">
+      <c r="E27" t="s">
         <v>1176</v>
       </c>
-      <c r="E27" t="s">
+      <c r="F27" t="s">
         <v>1177</v>
       </c>
-      <c r="F27" t="s">
+      <c r="G27" t="s">
         <v>1178</v>
       </c>
-      <c r="G27" t="s">
+      <c r="H27" t="s">
         <v>1179</v>
-      </c>
-      <c r="H27" t="s">
-        <v>1180</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.3">
@@ -6043,25 +6144,25 @@
         <v>46289</v>
       </c>
       <c r="B28" t="s">
+        <v>1180</v>
+      </c>
+      <c r="C28" t="s">
         <v>1181</v>
       </c>
-      <c r="C28" t="s">
+      <c r="D28" t="s">
         <v>1182</v>
       </c>
-      <c r="D28" t="s">
+      <c r="E28" t="s">
         <v>1183</v>
       </c>
-      <c r="E28" t="s">
+      <c r="F28" t="s">
         <v>1184</v>
       </c>
-      <c r="F28" t="s">
+      <c r="G28" t="s">
         <v>1185</v>
       </c>
-      <c r="G28" t="s">
-        <v>1186</v>
-      </c>
       <c r="H28" t="s">
-        <v>1166</v>
+        <v>1165</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.3">
@@ -6069,25 +6170,25 @@
         <v>46289</v>
       </c>
       <c r="B29" t="s">
+        <v>1186</v>
+      </c>
+      <c r="C29" t="s">
         <v>1187</v>
       </c>
-      <c r="C29" t="s">
+      <c r="D29" t="s">
         <v>1188</v>
       </c>
-      <c r="D29" t="s">
+      <c r="E29" t="s">
         <v>1189</v>
       </c>
-      <c r="E29" t="s">
+      <c r="F29" t="s">
         <v>1190</v>
       </c>
-      <c r="F29" t="s">
+      <c r="G29" t="s">
         <v>1191</v>
       </c>
-      <c r="G29" t="s">
-        <v>1192</v>
-      </c>
       <c r="H29" t="s">
-        <v>1166</v>
+        <v>1165</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.3">
@@ -6095,25 +6196,25 @@
         <v>46289</v>
       </c>
       <c r="B30" t="s">
+        <v>1192</v>
+      </c>
+      <c r="C30" t="s">
         <v>1193</v>
       </c>
-      <c r="C30" t="s">
+      <c r="D30" t="s">
         <v>1194</v>
       </c>
-      <c r="D30" t="s">
+      <c r="E30" t="s">
         <v>1195</v>
       </c>
-      <c r="E30" t="s">
+      <c r="F30" t="s">
         <v>1196</v>
       </c>
-      <c r="F30" t="s">
+      <c r="G30" t="s">
         <v>1197</v>
       </c>
-      <c r="G30" t="s">
+      <c r="H30" t="s">
         <v>1198</v>
-      </c>
-      <c r="H30" t="s">
-        <v>1199</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.3">
@@ -6121,25 +6222,103 @@
         <v>46289</v>
       </c>
       <c r="B31" t="s">
+        <v>1199</v>
+      </c>
+      <c r="C31" t="s">
         <v>1200</v>
       </c>
-      <c r="C31" t="s">
+      <c r="D31" t="s">
         <v>1201</v>
       </c>
-      <c r="D31" t="s">
+      <c r="E31" t="s">
         <v>1202</v>
       </c>
-      <c r="E31" t="s">
+      <c r="F31" t="s">
         <v>1203</v>
       </c>
-      <c r="F31" t="s">
+      <c r="G31" t="s">
         <v>1204</v>
       </c>
-      <c r="G31" t="s">
-        <v>1205</v>
-      </c>
       <c r="H31" t="s">
-        <v>1166</v>
+        <v>1165</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A32" s="12">
+        <v>46289</v>
+      </c>
+      <c r="B32" t="s">
+        <v>1222</v>
+      </c>
+      <c r="C32" t="s">
+        <v>1223</v>
+      </c>
+      <c r="D32" t="s">
+        <v>1224</v>
+      </c>
+      <c r="E32" t="s">
+        <v>1225</v>
+      </c>
+      <c r="F32" t="s">
+        <v>1226</v>
+      </c>
+      <c r="G32" t="s">
+        <v>1227</v>
+      </c>
+      <c r="H32" t="s">
+        <v>1228</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A33" s="12">
+        <v>46289</v>
+      </c>
+      <c r="B33" t="s">
+        <v>1229</v>
+      </c>
+      <c r="C33" t="s">
+        <v>1230</v>
+      </c>
+      <c r="D33" t="s">
+        <v>1231</v>
+      </c>
+      <c r="E33" t="s">
+        <v>1232</v>
+      </c>
+      <c r="F33" t="s">
+        <v>1233</v>
+      </c>
+      <c r="G33" t="s">
+        <v>1234</v>
+      </c>
+      <c r="H33" t="s">
+        <v>1228</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A34" s="12">
+        <v>46289</v>
+      </c>
+      <c r="B34" t="s">
+        <v>1235</v>
+      </c>
+      <c r="C34" t="s">
+        <v>1236</v>
+      </c>
+      <c r="D34" t="s">
+        <v>1237</v>
+      </c>
+      <c r="E34" t="s">
+        <v>1238</v>
+      </c>
+      <c r="F34" t="s">
+        <v>1239</v>
+      </c>
+      <c r="G34" t="s">
+        <v>1240</v>
+      </c>
+      <c r="H34" t="s">
+        <v>1241</v>
       </c>
     </row>
   </sheetData>
@@ -6495,10 +6674,10 @@
         <v>692</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>1097</v>
+        <v>1096</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>1121</v>
+        <v>1120</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="201.6" x14ac:dyDescent="0.3">
@@ -6509,10 +6688,10 @@
         <v>694</v>
       </c>
       <c r="C3" s="2" t="s">
+        <v>1121</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>1122</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>1123</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="201.6" x14ac:dyDescent="0.3">
@@ -6523,10 +6702,10 @@
         <v>696</v>
       </c>
       <c r="C4" s="2" t="s">
+        <v>1123</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>1124</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>1125</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="187.2" x14ac:dyDescent="0.3">
@@ -6537,10 +6716,10 @@
         <v>698</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>1124</v>
+        <v>1123</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>1126</v>
+        <v>1125</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="201.6" x14ac:dyDescent="0.3">
@@ -6551,10 +6730,10 @@
         <v>700</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>1124</v>
+        <v>1123</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>1127</v>
+        <v>1126</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="158.4" x14ac:dyDescent="0.3">
@@ -6565,10 +6744,10 @@
         <v>702</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>1124</v>
+        <v>1123</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>1128</v>
+        <v>1127</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="302.39999999999998" x14ac:dyDescent="0.3">
@@ -6579,10 +6758,10 @@
         <v>704</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>1122</v>
+        <v>1121</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>1129</v>
+        <v>1128</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="144" x14ac:dyDescent="0.3">
@@ -6593,10 +6772,10 @@
         <v>706</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>1097</v>
+        <v>1096</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>1130</v>
+        <v>1129</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="216" x14ac:dyDescent="0.3">
@@ -6607,10 +6786,10 @@
         <v>708</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>1122</v>
+        <v>1121</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>1131</v>
+        <v>1130</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="187.2" x14ac:dyDescent="0.3">
@@ -6621,10 +6800,10 @@
         <v>710</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>1124</v>
+        <v>1123</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>1132</v>
+        <v>1131</v>
       </c>
     </row>
   </sheetData>
@@ -6767,10 +6946,10 @@
         <v>739</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>1153</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" ht="172.8" x14ac:dyDescent="0.3">
+        <v>1152</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
         <v>740</v>
       </c>
@@ -6787,7 +6966,7 @@
         <v>741</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>1066</v>
+        <v>1242</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
@@ -6827,7 +7006,7 @@
         <v>750</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>1214</v>
+        <v>1212</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="201.6" x14ac:dyDescent="0.3">
@@ -6847,7 +7026,7 @@
         <v>754</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>1081</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="288" x14ac:dyDescent="0.3">
@@ -6867,7 +7046,7 @@
         <v>757</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>1213</v>
+        <v>1211</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="187.2" x14ac:dyDescent="0.3">
@@ -6887,7 +7066,7 @@
         <v>760</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>1212</v>
+        <v>1210</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="100.8" x14ac:dyDescent="0.3">
@@ -6927,7 +7106,7 @@
         <v>768</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>1211</v>
+        <v>1209</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="115.2" x14ac:dyDescent="0.3">
@@ -6947,7 +7126,7 @@
         <v>771</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>1210</v>
+        <v>1208</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="115.2" x14ac:dyDescent="0.3">
@@ -6967,10 +7146,10 @@
         <v>775</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>1209</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" ht="230.4" x14ac:dyDescent="0.3">
+        <v>1207</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="273.60000000000002" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
         <v>776</v>
       </c>
@@ -6987,7 +7166,7 @@
         <v>778</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>1208</v>
+        <v>1243</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="158.4" x14ac:dyDescent="0.3">
@@ -7007,7 +7186,7 @@
         <v>782</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>1207</v>
+        <v>1206</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="216" x14ac:dyDescent="0.3">
@@ -7027,15 +7206,15 @@
         <v>786</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>1206</v>
+        <v>1205</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>1220</v>
+        <v>1218</v>
       </c>
       <c r="B16" t="s">
-        <v>1221</v>
+        <v>1219</v>
       </c>
       <c r="C16" t="s">
         <v>737</v>
@@ -7044,10 +7223,10 @@
         <v>753</v>
       </c>
       <c r="E16" t="s">
-        <v>1222</v>
+        <v>1220</v>
       </c>
       <c r="F16" t="s">
-        <v>1223</v>
+        <v>1221</v>
       </c>
     </row>
     <row r="17" spans="1:1" ht="276" x14ac:dyDescent="0.3">
@@ -7249,7 +7428,7 @@
         <v>818</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>1074</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -7269,7 +7448,7 @@
         <v>103</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>1074</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -7289,7 +7468,7 @@
         <v>826</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>1074</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -7309,7 +7488,7 @@
         <v>829</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>1074</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -7329,7 +7508,7 @@
         <v>833</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>1074</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
@@ -7389,7 +7568,7 @@
         <v>152</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>1074</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -7409,7 +7588,7 @@
         <v>157</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>1074</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
@@ -7429,7 +7608,7 @@
         <v>849</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>1074</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="20" spans="1:6" ht="358.8" x14ac:dyDescent="0.3">
@@ -8204,7 +8383,7 @@
         <v>54</v>
       </c>
       <c r="J5" s="4" t="s">
-        <v>1154</v>
+        <v>1153</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
@@ -8550,7 +8729,7 @@
         <v>117</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>1073</v>
+        <v>1072</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Tracker: CHUNKS 14-16 verified against live production
First production verification - the push backlog was the standing blocker.
All 9 security headers present on live responses, all routes correct,
confidentiality audit clean on live HTML, SEO metadata complete, pages
2.5-4.5 KB gzipped, 2 JS islands.

Two findings, neither blocking: /styleguide is publicly reachable at 200,
and /about is sitemap-listed while noindex because its story is still
missing. Chunks stay Review - Lighthouse, rich-results, the /styleguide
deletion and the Sheet 13 re-run are what close them.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Raymund_Portfolio_PRD_Progress_Tracker.xlsx
+++ b/Raymund_Portfolio_PRD_Progress_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://gdslink-my.sharepoint.com/personal/raymund_bermudes_gdslinkasia_com/Documents/Documents/Rr/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="479" documentId="13_ncr:1_{E42DE829-FADD-499D-AC40-0688BE14A681}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BC2CE1DC-2AE1-4B04-8F07-DFB7DE1AF9E2}"/>
+  <xr:revisionPtr revIDLastSave="488" documentId="13_ncr:1_{E42DE829-FADD-499D-AC40-0688BE14A681}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CA2E6E54-499A-4F3D-9BFB-909845D52E4D}"/>
   <bookViews>
     <workbookView xWindow="2304" yWindow="2304" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1812" uniqueCount="1249">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1820" uniqueCount="1254">
   <si>
     <t>Portfolio Project PRD &amp; Progress Tracker</t>
   </si>
@@ -3785,6 +3785,21 @@
   </si>
   <si>
     <t>Only TWO content items remain: the About story (CG-15) and the CV PDF file (CG-04). Then push, verify CHUNKS 14-16 against production, delete /styleguide, re-run Sheet 13 recruiter test.</t>
+  </si>
+  <si>
+    <t>CHUNKS 14-16 verified against LIVE PRODUCTION for the first time</t>
+  </si>
+  <si>
+    <t>Everything to date is pushed and deployed - origin/main and HEAD both at 3185f70. This is the first time the QA chunks have been checked against production rather than localhost, which was the standing blocker. Both case studies are publicly live and the stage coverage strip renders 4 of 7 and 7 of 7 respectively.</t>
+  </si>
+  <si>
+    <t>SECURITY: all 9 headers present on live responses - CSP (script-src self, no unsafe-inline), HSTS w/ preload, X-Content-Type-Options, X-Frame-Options DENY, Referrer-Policy, Permissions-Policy, COOP, CORP. ROUTES: all 6 return 200, unknown path returns 404. CONFIDENTIALITY on live HTML: ctbc, c.t.b.c, sbc, appraisal, appraiser, bank, lender, taiwan all CLEAN. The only "philippin" hits are his own location, which is his data, not a client's. SEO: canonical, description, full OG block and JSON-LD on every page; sitemap lists 6 URLs, no trailing slashes; robots correct. WEIGHT: 2.5-4.5 KB gzipped HTML per page, far inside the 350 KB budget. JS: theme-init plus ThemeToggle everywhere, DeliveryThread on case studies only - 2 islands, inside the cap of 4.</t>
+  </si>
+  <si>
+    <t>TWO FINDINGS, neither blocking. (1) /styleguide returns 200 on production - it is a dev-only route that CLAUDE.md says to delete before launch and HANDOFF records as deliberately retained. It is excluded from the sitemap and Disallowed in robots, but it is publicly reachable and a recruiter could land on it. Decision needed: delete now or at true launch. (2) /about is listed in the sitemap while carrying noindex, because its story is still [CONTENT REQUIRED]. astro.config flags this exact case for re-check at CHUNK 16. It resolves itself the moment CG-15 lands; no action needed unless the story is deferred.</t>
+  </si>
+  <si>
+    <t>CHUNKS 14, 15 and 16 stay REVIEW, not Complete: no Lighthouse run against production yet, rich-results not tested, /styleguide not deleted, and the Sheet 13 recruiter test has not been re-run since the content landed. Those four are what closes them.</t>
   </si>
 </sst>
 </file>
@@ -4792,7 +4807,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -5376,45 +5391,71 @@
         <v>34</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A23" s="2"/>
-      <c r="B23" s="2" t="s">
+    <row r="23" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A23" s="10" t="s">
+        <v>1074</v>
+      </c>
+      <c r="B23" s="11" t="s">
         <v>141</v>
       </c>
-      <c r="C23" s="2"/>
-      <c r="D23" s="2" t="s">
-        <v>569</v>
-      </c>
-      <c r="E23" s="2"/>
-      <c r="F23" s="2"/>
-      <c r="G23" s="2" t="s">
-        <v>570</v>
-      </c>
-      <c r="H23" s="2" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="C23" s="11" t="s">
+        <v>1249</v>
+      </c>
+      <c r="D23" s="11" t="s">
+        <v>1250</v>
+      </c>
+      <c r="E23" s="11" t="s">
+        <v>1251</v>
+      </c>
+      <c r="F23" s="11" t="s">
+        <v>1252</v>
+      </c>
+      <c r="G23" s="11" t="s">
+        <v>1253</v>
+      </c>
+      <c r="H23" s="11" t="s">
+        <v>1073</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A24" s="2"/>
       <c r="B24" s="2" t="s">
-        <v>170</v>
+        <v>141</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" s="2" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="E24" s="2"/>
       <c r="F24" s="2"/>
       <c r="G24" s="2" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
       <c r="H24" s="2" t="s">
         <v>48</v>
       </c>
     </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A25" s="2"/>
+      <c r="B25" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="C25" s="2"/>
+      <c r="D25" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="E25" s="2"/>
+      <c r="F25" s="2"/>
+      <c r="G25" s="2" t="s">
+        <v>572</v>
+      </c>
+      <c r="H25" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="H2:H24" xr:uid="{00000000-0002-0000-0A00-000000000000}">
+    <dataValidation type="list" allowBlank="1" sqref="H2:H25" xr:uid="{00000000-0002-0000-0A00-000000000000}">
       <formula1>"Not Started,In Progress,Blocked,Review,Complete,On Hold"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
D34: retain /styleguide, defer CHUNK 16 closeout
Owner's call. The route still renders the whole design system and work is
ongoing, so deleting it now would cost more than it saves. Already excluded
from the sitemap and Disallowed in robots.

Recorded as a KNOWN, ACCEPTED exposure rather than an oversight: it returns
200 in production and must still be deleted before launch. D34 defers the
task, it does not cancel it.

HANDOFF next-actions rewritten: two content items remain - the About story
and the CV PDF file - and nothing else is blocked on code.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Raymund_Portfolio_PRD_Progress_Tracker.xlsx
+++ b/Raymund_Portfolio_PRD_Progress_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://gdslink-my.sharepoint.com/personal/raymund_bermudes_gdslinkasia_com/Documents/Documents/Rr/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="488" documentId="13_ncr:1_{E42DE829-FADD-499D-AC40-0688BE14A681}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CA2E6E54-499A-4F3D-9BFB-909845D52E4D}"/>
+  <xr:revisionPtr revIDLastSave="496" documentId="13_ncr:1_{E42DE829-FADD-499D-AC40-0688BE14A681}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0FE719F1-06BD-4697-A4AA-3410036F63FD}"/>
   <bookViews>
     <workbookView xWindow="2304" yWindow="2304" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1820" uniqueCount="1254">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1827" uniqueCount="1260">
   <si>
     <t>Portfolio Project PRD &amp; Progress Tracker</t>
   </si>
@@ -3800,6 +3800,24 @@
   </si>
   <si>
     <t>CHUNKS 14, 15 and 16 stay REVIEW, not Complete: no Lighthouse run against production yet, rich-results not tested, /styleguide not deleted, and the Sheet 13 recruiter test has not been re-run since the content landed. Those four are what closes them.</t>
+  </si>
+  <si>
+    <t>D34</t>
+  </si>
+  <si>
+    <t>/styleguide is RETAINED for now, and the CHUNK 16 closeout tasks are deferred</t>
+  </si>
+  <si>
+    <t>(a) Delete /styleguide now and run the CHUNK 16 closeout; (b) retain it and defer both until the remaining content lands</t>
+  </si>
+  <si>
+    <t>(b) Retain and defer</t>
+  </si>
+  <si>
+    <t>The route is still useful while work continues, and deleting it now would remove the one page that renders the whole design system while two content items are still outstanding. It is already excluded from the sitemap and Disallowed in robots.</t>
+  </si>
+  <si>
+    <t>Low, but it is a KNOWN EXPOSURE, not an oversight: /styleguide returns 200 in production and a visitor can reach it directly. Accepted deliberately. It MUST still be deleted before the site is treated as launched - this decision defers the task, it does not cancel it.</t>
   </si>
 </sst>
 </file>
@@ -5465,7 +5483,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
-  <dimension ref="A1:H34"/>
+  <dimension ref="A1:H35"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -6360,6 +6378,32 @@
       </c>
       <c r="H34" t="s">
         <v>1241</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A35" s="12">
+        <v>46289</v>
+      </c>
+      <c r="B35" t="s">
+        <v>1254</v>
+      </c>
+      <c r="C35" t="s">
+        <v>1255</v>
+      </c>
+      <c r="D35" t="s">
+        <v>1256</v>
+      </c>
+      <c r="E35" t="s">
+        <v>1257</v>
+      </c>
+      <c r="F35" t="s">
+        <v>1258</v>
+      </c>
+      <c r="G35" t="s">
+        <v>1259</v>
+      </c>
+      <c r="H35" t="s">
+        <v>1228</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
HANDOFF: one item left, verified live
About story confirmed live on production; /about is indexable. The only
[CONTENT REQUIRED] remaining anywhere on the site is the resume notice on
/contact, waiting on the PDF file itself.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Raymund_Portfolio_PRD_Progress_Tracker.xlsx
+++ b/Raymund_Portfolio_PRD_Progress_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://gdslink-my.sharepoint.com/personal/raymund_bermudes_gdslinkasia_com/Documents/Documents/Rr/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="496" documentId="13_ncr:1_{E42DE829-FADD-499D-AC40-0688BE14A681}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0FE719F1-06BD-4697-A4AA-3410036F63FD}"/>
+  <xr:revisionPtr revIDLastSave="505" documentId="13_ncr:1_{E42DE829-FADD-499D-AC40-0688BE14A681}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C738CC4C-CD49-4610-B873-D4B6713F144B}"/>
   <bookViews>
     <workbookView xWindow="2304" yWindow="2304" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1827" uniqueCount="1260">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1834" uniqueCount="1267">
   <si>
     <t>Portfolio Project PRD &amp; Progress Tracker</t>
   </si>
@@ -3703,9 +3703,6 @@
     <t>His own account, in his own voice. Prompts offered: how he got from Junior Android Developer to Solutions Analyst; what kind of problem he enjoys most; what he does differently from someone who only writes code. Rough notes are enough - Claude writes the prose from them.</t>
   </si>
   <si>
-    <t>Open - ADDED 2026-09-24. This gap was being rendered on /about as a visible [CONTENT REQUIRED] but was never tracked on this sheet. Nobody but the owner can write it; a generated version reads exactly like one.</t>
-  </si>
-  <si>
     <t>D31</t>
   </si>
   <si>
@@ -3818,6 +3815,30 @@
   </si>
   <si>
     <t>Low, but it is a KNOWN EXPOSURE, not an oversight: /styleguide returns 200 in production and a visitor can reach it directly. Accepted deliberately. It MUST still be deleted before the site is treated as launched - this decision defers the task, it does not cancel it.</t>
+  </si>
+  <si>
+    <t>D35</t>
+  </si>
+  <si>
+    <t>The About paragraph states what he DOES; it deliberately claims no motivation</t>
+  </si>
+  <si>
+    <t>(a) Write a motivation from the sentence he affirmed; (b) write a factual paragraph from sourced material only; (c) leave /about blocked until he supplies his own words</t>
+  </si>
+  <si>
+    <t>(b) Factual, sourced only</t>
+  </si>
+  <si>
+    <t>He delegated the choice: "ill let you decide on this". Option (a) was rejected because the only motivation available is a sentence CLAUDE offered as an example and he repeated back verbatim - the same provenance failure as the on-device storage line in case study 1, and this time Claude caused it by supplying the example. A feeling cannot be sourced. Option (c) would have left the last content gap open indefinitely over a sentence that is not required. Option (b) says what he does, which is checkable, and needs no attestation beyond answers he has already given.</t>
+  </si>
+  <si>
+    <t>Closes CG-15 and lifts /about's noindex, which also resolves the sitemap-lists-a-noindexed-page finding from the production audit. The clause-by-clause source mapping is written into src/pages/about.astro above the string, so a future edit cannot quietly loosen it. If he later supplies the motivation in his own words it belongs as a FOURTH sentence, not as a rewrite of the three.</t>
+  </si>
+  <si>
+    <t>DELEGATED by owner, DECIDED by Claude 2026-09-24</t>
+  </si>
+  <si>
+    <t>CLOSED 2026-09-24 (D35) - written from sourced material only. No motivation is claimed: the only one available was a Claude-supplied example he repeated back, so it was left out rather than published. Every clause traces to his CV or to an answer he gave, and the mapping is recorded in the page source. /about is now indexable.</t>
   </si>
 </sst>
 </file>
@@ -5391,19 +5412,19 @@
         <v>39</v>
       </c>
       <c r="C22" s="11" t="s">
+        <v>1243</v>
+      </c>
+      <c r="D22" s="11" t="s">
         <v>1244</v>
       </c>
-      <c r="D22" s="11" t="s">
+      <c r="E22" s="11" t="s">
         <v>1245</v>
       </c>
-      <c r="E22" s="11" t="s">
+      <c r="F22" s="11" t="s">
         <v>1246</v>
       </c>
-      <c r="F22" s="11" t="s">
+      <c r="G22" s="11" t="s">
         <v>1247</v>
-      </c>
-      <c r="G22" s="11" t="s">
-        <v>1248</v>
       </c>
       <c r="H22" s="11" t="s">
         <v>34</v>
@@ -5417,19 +5438,19 @@
         <v>141</v>
       </c>
       <c r="C23" s="11" t="s">
+        <v>1248</v>
+      </c>
+      <c r="D23" s="11" t="s">
         <v>1249</v>
       </c>
-      <c r="D23" s="11" t="s">
+      <c r="E23" s="11" t="s">
         <v>1250</v>
       </c>
-      <c r="E23" s="11" t="s">
+      <c r="F23" s="11" t="s">
         <v>1251</v>
       </c>
-      <c r="F23" s="11" t="s">
+      <c r="G23" s="11" t="s">
         <v>1252</v>
-      </c>
-      <c r="G23" s="11" t="s">
-        <v>1253</v>
       </c>
       <c r="H23" s="11" t="s">
         <v>1073</v>
@@ -5483,7 +5504,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
-  <dimension ref="A1:H35"/>
+  <dimension ref="A1:H36"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -6307,25 +6328,25 @@
         <v>46289</v>
       </c>
       <c r="B32" t="s">
+        <v>1221</v>
+      </c>
+      <c r="C32" t="s">
         <v>1222</v>
       </c>
-      <c r="C32" t="s">
+      <c r="D32" t="s">
         <v>1223</v>
       </c>
-      <c r="D32" t="s">
+      <c r="E32" t="s">
         <v>1224</v>
       </c>
-      <c r="E32" t="s">
+      <c r="F32" t="s">
         <v>1225</v>
       </c>
-      <c r="F32" t="s">
+      <c r="G32" t="s">
         <v>1226</v>
       </c>
-      <c r="G32" t="s">
+      <c r="H32" t="s">
         <v>1227</v>
-      </c>
-      <c r="H32" t="s">
-        <v>1228</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.3">
@@ -6333,25 +6354,25 @@
         <v>46289</v>
       </c>
       <c r="B33" t="s">
+        <v>1228</v>
+      </c>
+      <c r="C33" t="s">
         <v>1229</v>
       </c>
-      <c r="C33" t="s">
+      <c r="D33" t="s">
         <v>1230</v>
       </c>
-      <c r="D33" t="s">
+      <c r="E33" t="s">
         <v>1231</v>
       </c>
-      <c r="E33" t="s">
+      <c r="F33" t="s">
         <v>1232</v>
       </c>
-      <c r="F33" t="s">
+      <c r="G33" t="s">
         <v>1233</v>
       </c>
-      <c r="G33" t="s">
-        <v>1234</v>
-      </c>
       <c r="H33" t="s">
-        <v>1228</v>
+        <v>1227</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.3">
@@ -6359,25 +6380,25 @@
         <v>46289</v>
       </c>
       <c r="B34" t="s">
+        <v>1234</v>
+      </c>
+      <c r="C34" t="s">
         <v>1235</v>
       </c>
-      <c r="C34" t="s">
+      <c r="D34" t="s">
         <v>1236</v>
       </c>
-      <c r="D34" t="s">
+      <c r="E34" t="s">
         <v>1237</v>
       </c>
-      <c r="E34" t="s">
+      <c r="F34" t="s">
         <v>1238</v>
       </c>
-      <c r="F34" t="s">
+      <c r="G34" t="s">
         <v>1239</v>
       </c>
-      <c r="G34" t="s">
+      <c r="H34" t="s">
         <v>1240</v>
-      </c>
-      <c r="H34" t="s">
-        <v>1241</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.3">
@@ -6385,25 +6406,51 @@
         <v>46289</v>
       </c>
       <c r="B35" t="s">
+        <v>1253</v>
+      </c>
+      <c r="C35" t="s">
         <v>1254</v>
       </c>
-      <c r="C35" t="s">
+      <c r="D35" t="s">
         <v>1255</v>
       </c>
-      <c r="D35" t="s">
+      <c r="E35" t="s">
         <v>1256</v>
       </c>
-      <c r="E35" t="s">
+      <c r="F35" t="s">
         <v>1257</v>
       </c>
-      <c r="F35" t="s">
+      <c r="G35" t="s">
         <v>1258</v>
       </c>
-      <c r="G35" t="s">
+      <c r="H35" t="s">
+        <v>1227</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A36" s="12">
+        <v>46289</v>
+      </c>
+      <c r="B36" t="s">
         <v>1259</v>
       </c>
-      <c r="H35" t="s">
-        <v>1228</v>
+      <c r="C36" t="s">
+        <v>1260</v>
+      </c>
+      <c r="D36" t="s">
+        <v>1261</v>
+      </c>
+      <c r="E36" t="s">
+        <v>1262</v>
+      </c>
+      <c r="F36" t="s">
+        <v>1263</v>
+      </c>
+      <c r="G36" t="s">
+        <v>1264</v>
+      </c>
+      <c r="H36" t="s">
+        <v>1265</v>
       </c>
     </row>
   </sheetData>
@@ -7051,7 +7098,7 @@
         <v>741</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>1242</v>
+        <v>1241</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
@@ -7251,7 +7298,7 @@
         <v>778</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>1243</v>
+        <v>1242</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="158.4" x14ac:dyDescent="0.3">
@@ -7311,7 +7358,7 @@
         <v>1220</v>
       </c>
       <c r="F16" t="s">
-        <v>1221</v>
+        <v>1266</v>
       </c>
     </row>
     <row r="17" spans="1:1" ht="276" x14ac:dyDescent="0.3">

</xml_diff>